<commit_message>
Inclusão do rank de gillette supervisores, antes da valição dos supervisores 73 e 74
</commit_message>
<xml_diff>
--- a/CAMPANHAS_2026_08.xlsx
+++ b/CAMPANHAS_2026_08.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.0.37\Q-Tarkuss\TK_Producao\Planilhas\Metas P&amp;G\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Douglas\Desktop\CampanhasDunorte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D05F7FB-DA65-42E0-A793-B0406B86F635}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{304A19DB-EA45-40E9-A944-BCD2696FE101}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-59" yWindow="-16152" windowWidth="28740" windowHeight="15543" tabRatio="743" activeTab="8" xr2:uid="{D47B44F0-F69B-49A7-BD77-BBB35D25EC12}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" tabRatio="743" activeTab="4" xr2:uid="{D47B44F0-F69B-49A7-BD77-BBB35D25EC12}"/>
   </bookViews>
   <sheets>
     <sheet name="INDICADORES" sheetId="11" r:id="rId1"/>
@@ -20,15 +20,17 @@
     <sheet name="PREM_SUP" sheetId="14" r:id="rId5"/>
     <sheet name="RCA_DEVOL" sheetId="13" r:id="rId6"/>
     <sheet name="RCA_DEVOL_RANK" sheetId="17" r:id="rId7"/>
-    <sheet name="PREM_RCA" sheetId="12" r:id="rId8"/>
-    <sheet name="MIX_MIN" sheetId="18" r:id="rId9"/>
-    <sheet name="MIXMIN_GRUPO_PRODUTO" sheetId="19" r:id="rId10"/>
-    <sheet name="LISTING_PRODUTOS" sheetId="20" r:id="rId11"/>
+    <sheet name="SUP_DEVOL_RANK" sheetId="22" r:id="rId8"/>
+    <sheet name="PREM_RCA" sheetId="12" r:id="rId9"/>
+    <sheet name="MIX_MIN" sheetId="18" r:id="rId10"/>
+    <sheet name="MIXMIN_GRUPO_PRODUTO" sheetId="19" r:id="rId11"/>
+    <sheet name="LISTING_PRODUTOS" sheetId="20" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">MIX_MIN!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">MIXMIN_GRUPO_PRODUTO!$A$1:$E$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">PREM_RCA!$A$1:$G$460</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">MIX_MIN!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">MIXMIN_GRUPO_PRODUTO!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">PREM_RCA!$A$1:$G$460</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">PREM_SUP!$A$1:$F$97</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">RCA_DEVOL!$A$1:$L$77</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -52,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4923" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4935" uniqueCount="374">
   <si>
     <t>PANTENE KIT</t>
   </si>
@@ -2430,7 +2432,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A834EBCC-CC1C-4C8C-A5BE-5CBEA749A3A1}">
   <dimension ref="A1:I43"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="13.4" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.28515625" style="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="32.42578125" style="6" bestFit="1" customWidth="1"/>
@@ -2444,7 +2446,7 @@
     <col min="12" max="16384" width="8.85546875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>124</v>
       </c>
@@ -2464,7 +2466,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A2" s="63">
         <v>46235</v>
       </c>
@@ -2484,7 +2486,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A3" s="63">
         <v>46235</v>
       </c>
@@ -2504,7 +2506,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A4" s="63">
         <v>46235</v>
       </c>
@@ -2524,7 +2526,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A5" s="63">
         <v>46235</v>
       </c>
@@ -2544,7 +2546,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A6" s="63">
         <v>46235</v>
       </c>
@@ -2564,7 +2566,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A7" s="63">
         <v>46235</v>
       </c>
@@ -2584,7 +2586,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A8" s="63">
         <v>46235</v>
       </c>
@@ -2604,7 +2606,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A9" s="63">
         <v>46235</v>
       </c>
@@ -2624,7 +2626,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A10" s="63">
         <v>46235</v>
       </c>
@@ -2644,7 +2646,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A11" s="63">
         <v>46235</v>
       </c>
@@ -2664,7 +2666,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A12" s="63">
         <v>46235</v>
       </c>
@@ -2684,7 +2686,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A13" s="63">
         <v>46235</v>
       </c>
@@ -2704,7 +2706,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A14" s="63">
         <v>46235</v>
       </c>
@@ -2724,7 +2726,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A15" s="63">
         <v>46235</v>
       </c>
@@ -2744,7 +2746,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A16" s="63">
         <v>46235</v>
       </c>
@@ -2764,7 +2766,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A17" s="63">
         <v>46235</v>
       </c>
@@ -2784,7 +2786,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A18" s="63">
         <v>46235</v>
       </c>
@@ -2804,7 +2806,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A19" s="63">
         <v>46235</v>
       </c>
@@ -2824,7 +2826,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A20" s="63">
         <v>46235</v>
       </c>
@@ -2844,7 +2846,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A21" s="63">
         <v>46235</v>
       </c>
@@ -2864,7 +2866,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A22" s="63">
         <v>46235</v>
       </c>
@@ -2884,7 +2886,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A23" s="63">
         <v>46235</v>
       </c>
@@ -2904,7 +2906,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A24" s="63">
         <v>46235</v>
       </c>
@@ -2924,7 +2926,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A25" s="63">
         <v>46235</v>
       </c>
@@ -3004,7 +3006,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A29" s="63">
         <v>46235</v>
       </c>
@@ -3024,7 +3026,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A30" s="63">
         <v>46235</v>
       </c>
@@ -3044,7 +3046,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A31" s="63">
         <v>46235</v>
       </c>
@@ -3064,7 +3066,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A32" s="63">
         <v>46235</v>
       </c>
@@ -3084,7 +3086,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A33" s="63">
         <v>46235</v>
       </c>
@@ -3104,7 +3106,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A34" s="63">
         <v>46235</v>
       </c>
@@ -3124,7 +3126,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A35" s="63">
         <v>46235</v>
       </c>
@@ -3144,7 +3146,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A36" s="63">
         <v>46235</v>
       </c>
@@ -3164,7 +3166,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A37" s="63">
         <v>46235</v>
       </c>
@@ -3184,7 +3186,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A38" s="63">
         <v>46235</v>
       </c>
@@ -3204,7 +3206,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A39" s="63">
         <v>46235</v>
       </c>
@@ -3224,7 +3226,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A40" s="63">
         <v>46235</v>
       </c>
@@ -3267,7 +3269,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A42" s="63">
         <v>46235</v>
       </c>
@@ -3287,7 +3289,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" ht="13.35" x14ac:dyDescent="0.25">
       <c r="A43" s="63">
         <v>46235</v>
       </c>
@@ -3313,9 +3315,445 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A072811B-C283-42B7-8087-474598682C4A}">
+  <dimension ref="A1:J13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="109" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1" s="109" t="s">
+        <v>127</v>
+      </c>
+      <c r="C1" s="109" t="s">
+        <v>136</v>
+      </c>
+      <c r="D1" s="109" t="s">
+        <v>160</v>
+      </c>
+      <c r="E1" s="122" t="s">
+        <v>372</v>
+      </c>
+      <c r="F1" s="109" t="s">
+        <v>126</v>
+      </c>
+      <c r="G1" s="109" t="s">
+        <v>161</v>
+      </c>
+      <c r="H1" s="109" t="s">
+        <v>164</v>
+      </c>
+      <c r="I1" s="109" t="s">
+        <v>267</v>
+      </c>
+      <c r="J1" s="109" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="56">
+        <v>46235</v>
+      </c>
+      <c r="B2">
+        <v>73</v>
+      </c>
+      <c r="C2">
+        <v>7260</v>
+      </c>
+      <c r="D2">
+        <v>23398</v>
+      </c>
+      <c r="E2" s="1">
+        <v>3</v>
+      </c>
+      <c r="F2" t="s">
+        <v>274</v>
+      </c>
+      <c r="G2" t="s">
+        <v>275</v>
+      </c>
+      <c r="H2" t="s">
+        <v>276</v>
+      </c>
+      <c r="I2">
+        <v>66</v>
+      </c>
+      <c r="J2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="56">
+        <v>46235</v>
+      </c>
+      <c r="B3">
+        <v>105</v>
+      </c>
+      <c r="C3">
+        <v>1054</v>
+      </c>
+      <c r="D3">
+        <v>335122</v>
+      </c>
+      <c r="E3" s="1">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
+        <v>277</v>
+      </c>
+      <c r="G3" t="s">
+        <v>278</v>
+      </c>
+      <c r="H3" t="s">
+        <v>165</v>
+      </c>
+      <c r="I3">
+        <v>81</v>
+      </c>
+      <c r="J3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="56">
+        <v>46235</v>
+      </c>
+      <c r="B4">
+        <v>73</v>
+      </c>
+      <c r="C4">
+        <v>7358</v>
+      </c>
+      <c r="D4">
+        <v>315215</v>
+      </c>
+      <c r="E4" s="1">
+        <v>3</v>
+      </c>
+      <c r="F4" t="s">
+        <v>274</v>
+      </c>
+      <c r="G4" t="s">
+        <v>275</v>
+      </c>
+      <c r="H4" t="s">
+        <v>276</v>
+      </c>
+      <c r="I4">
+        <v>66</v>
+      </c>
+      <c r="J4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="56">
+        <v>46235</v>
+      </c>
+      <c r="B5">
+        <v>73</v>
+      </c>
+      <c r="C5">
+        <v>7351</v>
+      </c>
+      <c r="D5">
+        <v>41147</v>
+      </c>
+      <c r="E5" s="1">
+        <v>3</v>
+      </c>
+      <c r="F5" t="s">
+        <v>274</v>
+      </c>
+      <c r="G5" t="s">
+        <v>275</v>
+      </c>
+      <c r="H5" t="s">
+        <v>276</v>
+      </c>
+      <c r="I5">
+        <v>66</v>
+      </c>
+      <c r="J5">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="56">
+        <v>46235</v>
+      </c>
+      <c r="B6">
+        <v>60</v>
+      </c>
+      <c r="C6">
+        <v>6011</v>
+      </c>
+      <c r="D6">
+        <v>318518</v>
+      </c>
+      <c r="E6" s="1">
+        <v>1</v>
+      </c>
+      <c r="F6" t="s">
+        <v>277</v>
+      </c>
+      <c r="G6" t="s">
+        <v>275</v>
+      </c>
+      <c r="H6" t="s">
+        <v>279</v>
+      </c>
+      <c r="I6">
+        <v>85</v>
+      </c>
+      <c r="J6">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="56">
+        <v>46235</v>
+      </c>
+      <c r="B7">
+        <v>73</v>
+      </c>
+      <c r="C7">
+        <v>7358</v>
+      </c>
+      <c r="D7">
+        <v>302240</v>
+      </c>
+      <c r="E7" s="1">
+        <v>3</v>
+      </c>
+      <c r="F7" t="s">
+        <v>274</v>
+      </c>
+      <c r="G7" t="s">
+        <v>275</v>
+      </c>
+      <c r="H7" t="s">
+        <v>276</v>
+      </c>
+      <c r="I7">
+        <v>66</v>
+      </c>
+      <c r="J7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="56">
+        <v>46235</v>
+      </c>
+      <c r="B8">
+        <v>73</v>
+      </c>
+      <c r="C8">
+        <v>7350</v>
+      </c>
+      <c r="D8">
+        <v>28477</v>
+      </c>
+      <c r="E8" s="1">
+        <v>3</v>
+      </c>
+      <c r="F8" t="s">
+        <v>274</v>
+      </c>
+      <c r="G8" t="s">
+        <v>275</v>
+      </c>
+      <c r="H8" t="s">
+        <v>276</v>
+      </c>
+      <c r="I8">
+        <v>66</v>
+      </c>
+      <c r="J8">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="56">
+        <v>46235</v>
+      </c>
+      <c r="B9">
+        <v>60</v>
+      </c>
+      <c r="C9">
+        <v>222</v>
+      </c>
+      <c r="D9">
+        <v>31536</v>
+      </c>
+      <c r="E9" s="1">
+        <v>1</v>
+      </c>
+      <c r="F9" t="s">
+        <v>280</v>
+      </c>
+      <c r="G9" t="s">
+        <v>275</v>
+      </c>
+      <c r="H9" t="s">
+        <v>281</v>
+      </c>
+      <c r="I9">
+        <v>87</v>
+      </c>
+      <c r="J9">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="56">
+        <v>46235</v>
+      </c>
+      <c r="B10">
+        <v>60</v>
+      </c>
+      <c r="C10">
+        <v>6011</v>
+      </c>
+      <c r="D10">
+        <v>17367</v>
+      </c>
+      <c r="E10" s="1">
+        <v>1</v>
+      </c>
+      <c r="F10" t="s">
+        <v>277</v>
+      </c>
+      <c r="G10" t="s">
+        <v>275</v>
+      </c>
+      <c r="H10" t="s">
+        <v>276</v>
+      </c>
+      <c r="I10">
+        <v>61</v>
+      </c>
+      <c r="J10">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="120">
+        <v>46235</v>
+      </c>
+      <c r="B11" s="109">
+        <v>60</v>
+      </c>
+      <c r="C11" s="109">
+        <v>222</v>
+      </c>
+      <c r="D11" s="109">
+        <v>334788</v>
+      </c>
+      <c r="E11" s="123">
+        <v>1</v>
+      </c>
+      <c r="F11" s="109" t="s">
+        <v>280</v>
+      </c>
+      <c r="G11" s="109" t="s">
+        <v>275</v>
+      </c>
+      <c r="H11" s="109" t="s">
+        <v>281</v>
+      </c>
+      <c r="I11" s="109">
+        <v>87</v>
+      </c>
+      <c r="J11">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="120">
+        <v>46235</v>
+      </c>
+      <c r="B12" s="109">
+        <v>73</v>
+      </c>
+      <c r="C12" s="109">
+        <v>7506</v>
+      </c>
+      <c r="D12" s="109">
+        <v>334788</v>
+      </c>
+      <c r="E12" s="123">
+        <v>3</v>
+      </c>
+      <c r="F12" s="109" t="s">
+        <v>277</v>
+      </c>
+      <c r="G12" s="109" t="s">
+        <v>275</v>
+      </c>
+      <c r="H12" s="109" t="s">
+        <v>281</v>
+      </c>
+      <c r="I12" s="109">
+        <v>84</v>
+      </c>
+      <c r="J12">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="56">
+        <v>46235</v>
+      </c>
+      <c r="B13">
+        <v>105</v>
+      </c>
+      <c r="C13">
+        <v>6026</v>
+      </c>
+      <c r="D13">
+        <v>23492</v>
+      </c>
+      <c r="E13" s="1">
+        <v>1</v>
+      </c>
+      <c r="F13" t="s">
+        <v>280</v>
+      </c>
+      <c r="G13" t="s">
+        <v>278</v>
+      </c>
+      <c r="H13" t="s">
+        <v>165</v>
+      </c>
+      <c r="I13">
+        <v>89</v>
+      </c>
+      <c r="J13">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G1" xr:uid="{A072811B-C283-42B7-8087-474598682C4A}"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4ABB38E8-AF8A-4AA5-92BC-CEE3591DE8B5}">
   <dimension ref="A1:I976"/>
-  <sheetFormatPr defaultColWidth="17.28515625" defaultRowHeight="14.85" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="17.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
@@ -22224,10 +22662,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C51E02B-D0E1-436A-84F6-32F7AA1D457D}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="14.85" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.5703125" bestFit="1" customWidth="1"/>
@@ -22380,7 +22818,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89A3111D-85BC-4040-B044-61A701C77797}">
   <dimension ref="A1:G25"/>
-  <sheetFormatPr defaultRowHeight="14.85" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -22737,7 +23175,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65708516-ECBE-4FB0-A98C-B51C702A6091}">
   <dimension ref="A1:G22"/>
-  <sheetFormatPr defaultRowHeight="14.85" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -22942,7 +23380,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12442671-B67A-4EA2-9EB6-62409CEC93AE}">
   <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultRowHeight="14.85" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.28515625" style="56" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.28515625" bestFit="1" customWidth="1"/>
@@ -23324,7 +23762,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C0A85DA-C87F-4499-B15D-79B66D26946C}">
   <dimension ref="A1:F97"/>
-  <sheetFormatPr defaultRowHeight="14.85" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" style="56" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -25236,6 +25674,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F97" xr:uid="{0C0A85DA-C87F-4499-B15D-79B66D26946C}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
@@ -25243,7 +25682,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85269CFA-80F1-47F8-8ED0-33C5EDBA1395}">
   <dimension ref="A1:M77"/>
-  <sheetFormatPr defaultColWidth="18.28515625" defaultRowHeight="14.85" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="18.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" style="56"/>
     <col min="3" max="3" width="18.28515625" style="112"/>
@@ -25252,7 +25691,7 @@
     <col min="9" max="9" width="18.28515625" style="112"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="21.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="55" t="s">
         <v>124</v>
       </c>
@@ -25284,7 +25723,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A2" s="63">
         <v>46235</v>
       </c>
@@ -25322,7 +25761,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A3" s="63">
         <v>46235</v>
       </c>
@@ -25360,7 +25799,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A4" s="63">
         <v>46235</v>
       </c>
@@ -25398,7 +25837,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A5" s="63">
         <v>46235</v>
       </c>
@@ -25436,7 +25875,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A6" s="63">
         <v>46235</v>
       </c>
@@ -25474,7 +25913,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A7" s="63">
         <v>46235</v>
       </c>
@@ -25512,7 +25951,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A8" s="63">
         <v>46235</v>
       </c>
@@ -25550,7 +25989,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A9" s="63">
         <v>46235</v>
       </c>
@@ -25588,7 +26027,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A10" s="63">
         <v>46235</v>
       </c>
@@ -25626,7 +26065,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A11" s="63">
         <v>46235</v>
       </c>
@@ -25664,7 +26103,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A12" s="63">
         <v>46235</v>
       </c>
@@ -25702,7 +26141,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A13" s="63">
         <v>46235</v>
       </c>
@@ -25740,7 +26179,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A14" s="63">
         <v>46235</v>
       </c>
@@ -25778,7 +26217,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A15" s="63">
         <v>46235</v>
       </c>
@@ -25816,7 +26255,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A16" s="63">
         <v>46235</v>
       </c>
@@ -25854,7 +26293,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A17" s="63">
         <v>46235</v>
       </c>
@@ -25892,7 +26331,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A18" s="63">
         <v>46235</v>
       </c>
@@ -25930,7 +26369,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A19" s="63">
         <v>46235</v>
       </c>
@@ -25968,7 +26407,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A20" s="63">
         <v>46235</v>
       </c>
@@ -26006,7 +26445,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A21" s="63">
         <v>46235</v>
       </c>
@@ -26044,7 +26483,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A22" s="63">
         <v>46235</v>
       </c>
@@ -26082,7 +26521,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A23" s="63">
         <v>46235</v>
       </c>
@@ -26120,7 +26559,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A24" s="63">
         <v>46235</v>
       </c>
@@ -26158,7 +26597,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A25" s="63">
         <v>46235</v>
       </c>
@@ -26196,7 +26635,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A26" s="63">
         <v>46235</v>
       </c>
@@ -26234,7 +26673,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A27" s="63">
         <v>46235</v>
       </c>
@@ -26272,7 +26711,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A28" s="63">
         <v>46235</v>
       </c>
@@ -26310,7 +26749,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A29" s="63">
         <v>46235</v>
       </c>
@@ -26348,7 +26787,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A30" s="63">
         <v>46235</v>
       </c>
@@ -26386,7 +26825,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A31" s="63">
         <v>46235</v>
       </c>
@@ -26424,7 +26863,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A32" s="63">
         <v>46235</v>
       </c>
@@ -26462,7 +26901,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A33" s="63">
         <v>46235</v>
       </c>
@@ -26500,7 +26939,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A34" s="63">
         <v>46235</v>
       </c>
@@ -26538,7 +26977,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A35" s="63">
         <v>46235</v>
       </c>
@@ -26576,7 +27015,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A36" s="63">
         <v>46235</v>
       </c>
@@ -26614,7 +27053,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A37" s="63">
         <v>46235</v>
       </c>
@@ -26652,7 +27091,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A38" s="63">
         <v>46235</v>
       </c>
@@ -26690,7 +27129,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A39" s="63">
         <v>46235</v>
       </c>
@@ -26728,7 +27167,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:12" ht="14.85" x14ac:dyDescent="0.25">
       <c r="A40" s="63">
         <v>46235</v>
       </c>
@@ -28183,7 +28622,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F74CCC6-2C08-4F87-9FD8-B26290A9CCF6}">
   <dimension ref="A1:E77"/>
-  <sheetFormatPr defaultRowHeight="14.85" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.7109375" style="56" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.140625" style="112" bestFit="1" customWidth="1"/>
@@ -29470,9 +29909,164 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1AD0E48-0BC5-4455-AFCC-26874437F8A8}">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" style="56" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.140625" style="112" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="51.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="120" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1" s="109" t="s">
+        <v>127</v>
+      </c>
+      <c r="C1" s="121" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="56">
+        <v>46235</v>
+      </c>
+      <c r="B2">
+        <v>29</v>
+      </c>
+      <c r="C2" s="112">
+        <v>1.15E-2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="56">
+        <v>46235</v>
+      </c>
+      <c r="B3">
+        <v>33</v>
+      </c>
+      <c r="C3" s="112">
+        <v>1.15E-2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="56">
+        <v>46235</v>
+      </c>
+      <c r="B4">
+        <v>34</v>
+      </c>
+      <c r="C4" s="112">
+        <v>5.7499999999999999E-3</v>
+      </c>
+      <c r="D4" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="56">
+        <v>46235</v>
+      </c>
+      <c r="B5">
+        <v>39</v>
+      </c>
+      <c r="C5" s="112">
+        <v>1.15E-2</v>
+      </c>
+      <c r="D5" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="56">
+        <v>46235</v>
+      </c>
+      <c r="B6">
+        <v>60</v>
+      </c>
+      <c r="C6" s="112">
+        <v>5.7499999999999999E-3</v>
+      </c>
+      <c r="D6" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="56">
+        <v>46235</v>
+      </c>
+      <c r="B7">
+        <v>75</v>
+      </c>
+      <c r="C7" s="112">
+        <v>1.15E-2</v>
+      </c>
+      <c r="D7" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="56">
+        <v>46235</v>
+      </c>
+      <c r="B8">
+        <v>76</v>
+      </c>
+      <c r="C8" s="112">
+        <v>1.15E-2</v>
+      </c>
+      <c r="D8" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="56">
+        <v>46235</v>
+      </c>
+      <c r="B9">
+        <v>105</v>
+      </c>
+      <c r="C9" s="112">
+        <v>5.7499999999999999E-3</v>
+      </c>
+      <c r="D9" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="56">
+        <v>46235</v>
+      </c>
+      <c r="B10">
+        <v>7374</v>
+      </c>
+      <c r="C10" s="112">
+        <v>5.7499999999999999E-3</v>
+      </c>
+      <c r="D10" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D16" s="56"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C42F608-3DF2-4BEF-9ABA-200CB43F9E80}">
   <dimension ref="A1:G460"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="11.9" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.7109375" style="78" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.85546875" style="51" bestFit="1" customWidth="1"/>
@@ -39790,440 +40384,4 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A072811B-C283-42B7-8087-474598682C4A}">
-  <dimension ref="A1:J13"/>
-  <sheetFormatPr defaultRowHeight="14.85" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="109" t="s">
-        <v>124</v>
-      </c>
-      <c r="B1" s="109" t="s">
-        <v>127</v>
-      </c>
-      <c r="C1" s="109" t="s">
-        <v>136</v>
-      </c>
-      <c r="D1" s="109" t="s">
-        <v>160</v>
-      </c>
-      <c r="E1" s="122" t="s">
-        <v>372</v>
-      </c>
-      <c r="F1" s="109" t="s">
-        <v>126</v>
-      </c>
-      <c r="G1" s="109" t="s">
-        <v>161</v>
-      </c>
-      <c r="H1" s="109" t="s">
-        <v>164</v>
-      </c>
-      <c r="I1" s="109" t="s">
-        <v>267</v>
-      </c>
-      <c r="J1" s="109" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="56">
-        <v>46235</v>
-      </c>
-      <c r="B2">
-        <v>73</v>
-      </c>
-      <c r="C2">
-        <v>7260</v>
-      </c>
-      <c r="D2">
-        <v>23398</v>
-      </c>
-      <c r="E2" s="1">
-        <v>3</v>
-      </c>
-      <c r="F2" t="s">
-        <v>274</v>
-      </c>
-      <c r="G2" t="s">
-        <v>275</v>
-      </c>
-      <c r="H2" t="s">
-        <v>276</v>
-      </c>
-      <c r="I2">
-        <v>66</v>
-      </c>
-      <c r="J2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="56">
-        <v>46235</v>
-      </c>
-      <c r="B3">
-        <v>105</v>
-      </c>
-      <c r="C3">
-        <v>1054</v>
-      </c>
-      <c r="D3">
-        <v>335122</v>
-      </c>
-      <c r="E3" s="1">
-        <v>1</v>
-      </c>
-      <c r="F3" t="s">
-        <v>277</v>
-      </c>
-      <c r="G3" t="s">
-        <v>278</v>
-      </c>
-      <c r="H3" t="s">
-        <v>165</v>
-      </c>
-      <c r="I3">
-        <v>81</v>
-      </c>
-      <c r="J3">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="56">
-        <v>46235</v>
-      </c>
-      <c r="B4">
-        <v>73</v>
-      </c>
-      <c r="C4">
-        <v>7358</v>
-      </c>
-      <c r="D4">
-        <v>315215</v>
-      </c>
-      <c r="E4" s="1">
-        <v>3</v>
-      </c>
-      <c r="F4" t="s">
-        <v>274</v>
-      </c>
-      <c r="G4" t="s">
-        <v>275</v>
-      </c>
-      <c r="H4" t="s">
-        <v>276</v>
-      </c>
-      <c r="I4">
-        <v>66</v>
-      </c>
-      <c r="J4">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="56">
-        <v>46235</v>
-      </c>
-      <c r="B5">
-        <v>73</v>
-      </c>
-      <c r="C5">
-        <v>7351</v>
-      </c>
-      <c r="D5">
-        <v>41147</v>
-      </c>
-      <c r="E5" s="1">
-        <v>3</v>
-      </c>
-      <c r="F5" t="s">
-        <v>274</v>
-      </c>
-      <c r="G5" t="s">
-        <v>275</v>
-      </c>
-      <c r="H5" t="s">
-        <v>276</v>
-      </c>
-      <c r="I5">
-        <v>66</v>
-      </c>
-      <c r="J5">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="56">
-        <v>46235</v>
-      </c>
-      <c r="B6">
-        <v>60</v>
-      </c>
-      <c r="C6">
-        <v>6011</v>
-      </c>
-      <c r="D6">
-        <v>318518</v>
-      </c>
-      <c r="E6" s="1">
-        <v>1</v>
-      </c>
-      <c r="F6" t="s">
-        <v>277</v>
-      </c>
-      <c r="G6" t="s">
-        <v>275</v>
-      </c>
-      <c r="H6" t="s">
-        <v>279</v>
-      </c>
-      <c r="I6">
-        <v>85</v>
-      </c>
-      <c r="J6">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="56">
-        <v>46235</v>
-      </c>
-      <c r="B7">
-        <v>73</v>
-      </c>
-      <c r="C7">
-        <v>7358</v>
-      </c>
-      <c r="D7">
-        <v>302240</v>
-      </c>
-      <c r="E7" s="1">
-        <v>3</v>
-      </c>
-      <c r="F7" t="s">
-        <v>274</v>
-      </c>
-      <c r="G7" t="s">
-        <v>275</v>
-      </c>
-      <c r="H7" t="s">
-        <v>276</v>
-      </c>
-      <c r="I7">
-        <v>66</v>
-      </c>
-      <c r="J7">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="56">
-        <v>46235</v>
-      </c>
-      <c r="B8">
-        <v>73</v>
-      </c>
-      <c r="C8">
-        <v>7350</v>
-      </c>
-      <c r="D8">
-        <v>28477</v>
-      </c>
-      <c r="E8" s="1">
-        <v>3</v>
-      </c>
-      <c r="F8" t="s">
-        <v>274</v>
-      </c>
-      <c r="G8" t="s">
-        <v>275</v>
-      </c>
-      <c r="H8" t="s">
-        <v>276</v>
-      </c>
-      <c r="I8">
-        <v>66</v>
-      </c>
-      <c r="J8">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="56">
-        <v>46235</v>
-      </c>
-      <c r="B9">
-        <v>60</v>
-      </c>
-      <c r="C9">
-        <v>222</v>
-      </c>
-      <c r="D9">
-        <v>31536</v>
-      </c>
-      <c r="E9" s="1">
-        <v>1</v>
-      </c>
-      <c r="F9" t="s">
-        <v>280</v>
-      </c>
-      <c r="G9" t="s">
-        <v>275</v>
-      </c>
-      <c r="H9" t="s">
-        <v>281</v>
-      </c>
-      <c r="I9">
-        <v>87</v>
-      </c>
-      <c r="J9">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="56">
-        <v>46235</v>
-      </c>
-      <c r="B10">
-        <v>60</v>
-      </c>
-      <c r="C10">
-        <v>6011</v>
-      </c>
-      <c r="D10">
-        <v>17367</v>
-      </c>
-      <c r="E10" s="1">
-        <v>1</v>
-      </c>
-      <c r="F10" t="s">
-        <v>277</v>
-      </c>
-      <c r="G10" t="s">
-        <v>275</v>
-      </c>
-      <c r="H10" t="s">
-        <v>276</v>
-      </c>
-      <c r="I10">
-        <v>61</v>
-      </c>
-      <c r="J10">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="120">
-        <v>46235</v>
-      </c>
-      <c r="B11" s="109">
-        <v>60</v>
-      </c>
-      <c r="C11" s="109">
-        <v>222</v>
-      </c>
-      <c r="D11" s="109">
-        <v>334788</v>
-      </c>
-      <c r="E11" s="123">
-        <v>1</v>
-      </c>
-      <c r="F11" s="109" t="s">
-        <v>280</v>
-      </c>
-      <c r="G11" s="109" t="s">
-        <v>275</v>
-      </c>
-      <c r="H11" s="109" t="s">
-        <v>281</v>
-      </c>
-      <c r="I11" s="109">
-        <v>87</v>
-      </c>
-      <c r="J11">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="120">
-        <v>46235</v>
-      </c>
-      <c r="B12" s="109">
-        <v>73</v>
-      </c>
-      <c r="C12" s="109">
-        <v>7506</v>
-      </c>
-      <c r="D12" s="109">
-        <v>334788</v>
-      </c>
-      <c r="E12" s="123">
-        <v>3</v>
-      </c>
-      <c r="F12" s="109" t="s">
-        <v>277</v>
-      </c>
-      <c r="G12" s="109" t="s">
-        <v>275</v>
-      </c>
-      <c r="H12" s="109" t="s">
-        <v>281</v>
-      </c>
-      <c r="I12" s="109">
-        <v>84</v>
-      </c>
-      <c r="J12">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="56">
-        <v>46235</v>
-      </c>
-      <c r="B13">
-        <v>105</v>
-      </c>
-      <c r="C13">
-        <v>6026</v>
-      </c>
-      <c r="D13">
-        <v>23492</v>
-      </c>
-      <c r="E13" s="1">
-        <v>1</v>
-      </c>
-      <c r="F13" t="s">
-        <v>280</v>
-      </c>
-      <c r="G13" t="s">
-        <v>278</v>
-      </c>
-      <c r="H13" t="s">
-        <v>165</v>
-      </c>
-      <c r="I13">
-        <v>89</v>
-      </c>
-      <c r="J13">
-        <v>12</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:G1" xr:uid="{A072811B-C283-42B7-8087-474598682C4A}"/>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
 </file>
</xml_diff>